<commit_message>
Modifications du Diagramme Gantt
Reprogrammation de tâches et fonctionnalités terminées
</commit_message>
<xml_diff>
--- a/Gantt Mastermind.xlsx
+++ b/Gantt Mastermind.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28814"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10511"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://univbourgogne-my.sharepoint.com/personal/nathan_kubiez-develay_etu_u-bourgogne_fr/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dimitricourtoisrozelot/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF807036-D30D-4C45-A229-2EB3D963A7D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC224AFD-BE79-884E-A9F5-04A481AF39EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1120" yWindow="740" windowWidth="28280" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="42">
   <si>
     <t>Mastermind</t>
   </si>
@@ -154,12 +154,6 @@
     <t xml:space="preserve">generer une combinaison </t>
   </si>
   <si>
-    <t xml:space="preserve">afficher la ligne et la pallette </t>
-  </si>
-  <si>
-    <t>gestion des clic</t>
-  </si>
-  <si>
     <t>Verification de la combianaison/affichage dernier essai</t>
   </si>
   <si>
@@ -169,6 +163,15 @@
     <t>ajout d'un menu simple</t>
   </si>
   <si>
+    <t>afficher le nombre d'éssais</t>
+  </si>
+  <si>
+    <t>faire une fin</t>
+  </si>
+  <si>
+    <t>améliorer l'affichage des lignes validées</t>
+  </si>
+  <si>
     <t>ajout différent niveau de difficulté</t>
   </si>
   <si>
@@ -176,37 +179,13 @@
   </si>
   <si>
     <t>Améliorier l'esthétique</t>
-  </si>
-  <si>
-    <t>Class Line</t>
-  </si>
-  <si>
-    <t>Class DoneLineGestion</t>
-  </si>
-  <si>
-    <t>Class SceneGestion &amp; Scene</t>
-  </si>
-  <si>
-    <t>Class GameScene</t>
-  </si>
-  <si>
-    <t>Class MenuScene</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Class GameGestion </t>
-  </si>
-  <si>
-    <t>ajouter des niveaux de difficulté</t>
-  </si>
-  <si>
-    <t>ajouter des options (abandonner,....)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -247,6 +226,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -286,7 +270,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -436,7 +420,31 @@
       </left>
       <right/>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="9"/>
+      </right>
+      <top style="medium">
+        <color theme="9"/>
+      </top>
       <bottom style="medium">
+        <color theme="9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF00B050"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF00B050"/>
+      </top>
+      <bottom style="thin">
         <color rgb="FF00B050"/>
       </bottom>
       <diagonal/>
@@ -444,9 +452,52 @@
     <border>
       <left/>
       <right/>
-      <top/>
+      <top style="thin">
+        <color rgb="FF00B050"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF00B050"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF00B050"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF00B050"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF00B050"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF00B050"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF00B050"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF00B050"/>
+      </top>
       <bottom style="medium">
         <color rgb="FF00B050"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="9"/>
+      </right>
+      <top style="medium">
+        <color theme="9"/>
+      </top>
+      <bottom style="medium">
+        <color theme="9"/>
       </bottom>
       <diagonal/>
     </border>
@@ -454,7 +505,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -501,7 +552,34 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -513,12 +591,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -853,182 +928,182 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CX43"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <dimension ref="A1:CX67"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="19.5" customWidth="1"/>
     <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
     <col min="5" max="17" width="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="2.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="2.28515625" customWidth="1"/>
+    <col min="18" max="19" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="2.33203125" customWidth="1"/>
     <col min="21" max="21" width="2" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="2.42578125" customWidth="1"/>
+    <col min="22" max="23" width="2.5" customWidth="1"/>
     <col min="24" max="24" width="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="2.7109375" customWidth="1"/>
-    <col min="26" max="26" width="2.42578125" customWidth="1"/>
+    <col min="25" max="25" width="2.6640625" customWidth="1"/>
+    <col min="26" max="26" width="2.5" customWidth="1"/>
     <col min="27" max="47" width="3" bestFit="1" customWidth="1"/>
     <col min="48" max="50" width="2" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="2.1640625" bestFit="1" customWidth="1"/>
     <col min="52" max="52" width="2" bestFit="1" customWidth="1"/>
-    <col min="53" max="54" width="2.42578125" bestFit="1" customWidth="1"/>
+    <col min="53" max="54" width="2.5" bestFit="1" customWidth="1"/>
     <col min="55" max="56" width="2" bestFit="1" customWidth="1"/>
     <col min="57" max="78" width="3" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="2.1640625" bestFit="1" customWidth="1"/>
     <col min="80" max="80" width="2" bestFit="1" customWidth="1"/>
-    <col min="81" max="82" width="2.42578125" bestFit="1" customWidth="1"/>
+    <col min="81" max="82" width="2.5" bestFit="1" customWidth="1"/>
     <col min="83" max="85" width="2" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="2.1640625" bestFit="1" customWidth="1"/>
     <col min="87" max="87" width="2" bestFit="1" customWidth="1"/>
     <col min="88" max="102" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:102">
-      <c r="A1" s="29"/>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="29"/>
-      <c r="S1" s="29"/>
-      <c r="T1" s="29"/>
-      <c r="U1" s="29"/>
-      <c r="V1" s="29"/>
-      <c r="W1" s="29"/>
-      <c r="X1" s="29"/>
-      <c r="Y1" s="29"/>
-      <c r="Z1" s="29"/>
-      <c r="AA1" s="29"/>
-      <c r="AB1" s="29"/>
-      <c r="AC1" s="29"/>
-      <c r="AD1" s="29"/>
-      <c r="AE1" s="29"/>
-      <c r="AF1" s="29"/>
-      <c r="AG1" s="29"/>
-      <c r="AH1" s="29"/>
-      <c r="AI1" s="29"/>
-      <c r="AJ1" s="29"/>
-      <c r="AK1" s="29"/>
-      <c r="AL1" s="29"/>
-      <c r="AM1" s="29"/>
-      <c r="AN1" s="29"/>
-      <c r="AO1" s="29"/>
-      <c r="AP1" s="29"/>
-      <c r="AQ1" s="29"/>
-      <c r="AR1" s="29"/>
-      <c r="AS1" s="29"/>
-      <c r="AT1" s="29"/>
-      <c r="AU1" s="29"/>
-      <c r="AV1" s="29"/>
-      <c r="AW1" s="29"/>
-      <c r="AX1" s="29"/>
-      <c r="AY1" s="29"/>
-      <c r="AZ1" s="29"/>
-      <c r="BA1" s="29"/>
-      <c r="BB1" s="29"/>
-      <c r="BC1" s="29"/>
-      <c r="BD1" s="29"/>
-      <c r="BE1" s="29"/>
-      <c r="BF1" s="29"/>
-      <c r="BG1" s="29"/>
-      <c r="BH1" s="29"/>
-      <c r="BI1" s="29"/>
-      <c r="BJ1" s="29"/>
-      <c r="BK1" s="29"/>
-      <c r="BL1" s="29"/>
-      <c r="BM1" s="29"/>
-      <c r="BN1" s="29"/>
-      <c r="BO1" s="29"/>
-      <c r="BP1" s="29"/>
-      <c r="BQ1" s="29"/>
-      <c r="BR1" s="29"/>
-      <c r="BS1" s="29"/>
-      <c r="BT1" s="29"/>
-      <c r="BU1" s="29"/>
-      <c r="BV1" s="29"/>
-      <c r="BW1" s="29"/>
-      <c r="BX1" s="29"/>
-      <c r="BY1" s="29"/>
-      <c r="BZ1" s="29"/>
-      <c r="CA1" s="29"/>
-      <c r="CB1" s="29"/>
-      <c r="CC1" s="29"/>
-      <c r="CD1" s="29"/>
-      <c r="CE1" s="29"/>
-      <c r="CF1" s="29"/>
-      <c r="CG1" s="29"/>
-      <c r="CH1" s="29"/>
-      <c r="CI1" s="29"/>
-      <c r="CJ1" s="29"/>
-      <c r="CK1" s="29"/>
-      <c r="CL1" s="29"/>
-      <c r="CM1" s="29"/>
-      <c r="CN1" s="29"/>
-      <c r="CO1" s="29"/>
-      <c r="CP1" s="29"/>
-      <c r="CQ1" s="29"/>
-      <c r="CR1" s="29"/>
-      <c r="CS1" s="29"/>
-      <c r="CT1" s="29"/>
-      <c r="CU1" s="29"/>
-      <c r="CV1" s="29"/>
-      <c r="CW1" s="29"/>
-      <c r="CX1" s="29"/>
-    </row>
-    <row r="2" spans="1:102">
-      <c r="A2" s="29"/>
-      <c r="B2" s="28" t="s">
+    <row r="1" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="44"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
+      <c r="P1" s="44"/>
+      <c r="Q1" s="44"/>
+      <c r="R1" s="44"/>
+      <c r="S1" s="44"/>
+      <c r="T1" s="44"/>
+      <c r="U1" s="44"/>
+      <c r="V1" s="44"/>
+      <c r="W1" s="44"/>
+      <c r="X1" s="44"/>
+      <c r="Y1" s="44"/>
+      <c r="Z1" s="44"/>
+      <c r="AA1" s="44"/>
+      <c r="AB1" s="44"/>
+      <c r="AC1" s="44"/>
+      <c r="AD1" s="44"/>
+      <c r="AE1" s="44"/>
+      <c r="AF1" s="44"/>
+      <c r="AG1" s="44"/>
+      <c r="AH1" s="44"/>
+      <c r="AI1" s="44"/>
+      <c r="AJ1" s="44"/>
+      <c r="AK1" s="44"/>
+      <c r="AL1" s="44"/>
+      <c r="AM1" s="44"/>
+      <c r="AN1" s="44"/>
+      <c r="AO1" s="44"/>
+      <c r="AP1" s="44"/>
+      <c r="AQ1" s="44"/>
+      <c r="AR1" s="44"/>
+      <c r="AS1" s="44"/>
+      <c r="AT1" s="44"/>
+      <c r="AU1" s="44"/>
+      <c r="AV1" s="44"/>
+      <c r="AW1" s="44"/>
+      <c r="AX1" s="44"/>
+      <c r="AY1" s="44"/>
+      <c r="AZ1" s="44"/>
+      <c r="BA1" s="44"/>
+      <c r="BB1" s="44"/>
+      <c r="BC1" s="44"/>
+      <c r="BD1" s="44"/>
+      <c r="BE1" s="44"/>
+      <c r="BF1" s="44"/>
+      <c r="BG1" s="44"/>
+      <c r="BH1" s="44"/>
+      <c r="BI1" s="44"/>
+      <c r="BJ1" s="44"/>
+      <c r="BK1" s="44"/>
+      <c r="BL1" s="44"/>
+      <c r="BM1" s="44"/>
+      <c r="BN1" s="44"/>
+      <c r="BO1" s="44"/>
+      <c r="BP1" s="44"/>
+      <c r="BQ1" s="44"/>
+      <c r="BR1" s="44"/>
+      <c r="BS1" s="44"/>
+      <c r="BT1" s="44"/>
+      <c r="BU1" s="44"/>
+      <c r="BV1" s="44"/>
+      <c r="BW1" s="44"/>
+      <c r="BX1" s="44"/>
+      <c r="BY1" s="44"/>
+      <c r="BZ1" s="44"/>
+      <c r="CA1" s="44"/>
+      <c r="CB1" s="44"/>
+      <c r="CC1" s="44"/>
+      <c r="CD1" s="44"/>
+      <c r="CE1" s="44"/>
+      <c r="CF1" s="44"/>
+      <c r="CG1" s="44"/>
+      <c r="CH1" s="44"/>
+      <c r="CI1" s="44"/>
+      <c r="CJ1" s="44"/>
+      <c r="CK1" s="44"/>
+      <c r="CL1" s="44"/>
+      <c r="CM1" s="44"/>
+      <c r="CN1" s="44"/>
+      <c r="CO1" s="44"/>
+      <c r="CP1" s="44"/>
+      <c r="CQ1" s="44"/>
+      <c r="CR1" s="44"/>
+      <c r="CS1" s="44"/>
+      <c r="CT1" s="44"/>
+      <c r="CU1" s="44"/>
+      <c r="CV1" s="44"/>
+      <c r="CW1" s="44"/>
+      <c r="CX1" s="44"/>
+    </row>
+    <row r="2" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="44"/>
+      <c r="B2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28" t="s">
+      <c r="C2" s="42"/>
+      <c r="D2" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
       <c r="I2" s="1"/>
       <c r="J2" s="4"/>
-      <c r="K2" s="31" t="s">
+      <c r="K2" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
       <c r="O2" s="2"/>
-      <c r="P2" s="28" t="s">
+      <c r="P2" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="Q2" s="28"/>
-      <c r="R2" s="28"/>
+      <c r="Q2" s="42"/>
+      <c r="R2" s="42"/>
       <c r="S2" s="1"/>
       <c r="T2" s="5"/>
-      <c r="U2" s="28" t="s">
+      <c r="U2" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="V2" s="28"/>
-      <c r="W2" s="28"/>
+      <c r="V2" s="42"/>
+      <c r="W2" s="42"/>
       <c r="X2" s="1"/>
       <c r="Y2" s="3"/>
       <c r="Z2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:102" ht="15" customHeight="1">
-      <c r="A3" s="29"/>
+    <row r="3" spans="1:102" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="44"/>
       <c r="B3" s="10" t="s">
         <v>6</v>
       </c>
@@ -1038,119 +1113,119 @@
       <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="E3" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
-      <c r="K3" s="28"/>
-      <c r="L3" s="28"/>
-      <c r="M3" s="28"/>
-      <c r="N3" s="28"/>
-      <c r="O3" s="28"/>
-      <c r="P3" s="28"/>
-      <c r="Q3" s="28"/>
-      <c r="R3" s="28" t="s">
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="42"/>
+      <c r="M3" s="42"/>
+      <c r="N3" s="42"/>
+      <c r="O3" s="42"/>
+      <c r="P3" s="42"/>
+      <c r="Q3" s="42"/>
+      <c r="R3" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="S3" s="28"/>
-      <c r="T3" s="28"/>
-      <c r="U3" s="28"/>
-      <c r="V3" s="28"/>
-      <c r="W3" s="28"/>
-      <c r="X3" s="28"/>
-      <c r="Y3" s="28"/>
-      <c r="Z3" s="28"/>
-      <c r="AA3" s="28"/>
-      <c r="AB3" s="28"/>
-      <c r="AC3" s="28"/>
-      <c r="AD3" s="28"/>
-      <c r="AE3" s="28"/>
-      <c r="AF3" s="28"/>
-      <c r="AG3" s="28"/>
-      <c r="AH3" s="28"/>
-      <c r="AI3" s="28"/>
-      <c r="AJ3" s="28"/>
-      <c r="AK3" s="28"/>
-      <c r="AL3" s="28"/>
-      <c r="AM3" s="28"/>
-      <c r="AN3" s="28"/>
-      <c r="AO3" s="28"/>
-      <c r="AP3" s="28"/>
-      <c r="AQ3" s="28"/>
-      <c r="AR3" s="28"/>
-      <c r="AS3" s="28"/>
-      <c r="AT3" s="28"/>
-      <c r="AU3" s="28"/>
-      <c r="AV3" s="28" t="s">
+      <c r="S3" s="42"/>
+      <c r="T3" s="42"/>
+      <c r="U3" s="42"/>
+      <c r="V3" s="42"/>
+      <c r="W3" s="42"/>
+      <c r="X3" s="42"/>
+      <c r="Y3" s="42"/>
+      <c r="Z3" s="42"/>
+      <c r="AA3" s="42"/>
+      <c r="AB3" s="42"/>
+      <c r="AC3" s="42"/>
+      <c r="AD3" s="42"/>
+      <c r="AE3" s="42"/>
+      <c r="AF3" s="42"/>
+      <c r="AG3" s="42"/>
+      <c r="AH3" s="42"/>
+      <c r="AI3" s="42"/>
+      <c r="AJ3" s="42"/>
+      <c r="AK3" s="42"/>
+      <c r="AL3" s="42"/>
+      <c r="AM3" s="42"/>
+      <c r="AN3" s="42"/>
+      <c r="AO3" s="42"/>
+      <c r="AP3" s="42"/>
+      <c r="AQ3" s="42"/>
+      <c r="AR3" s="42"/>
+      <c r="AS3" s="42"/>
+      <c r="AT3" s="42"/>
+      <c r="AU3" s="42"/>
+      <c r="AV3" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="AW3" s="28"/>
-      <c r="AX3" s="28"/>
-      <c r="AY3" s="28"/>
-      <c r="AZ3" s="28"/>
-      <c r="BA3" s="28"/>
-      <c r="BB3" s="28"/>
-      <c r="BC3" s="28"/>
-      <c r="BD3" s="28"/>
-      <c r="BE3" s="28"/>
-      <c r="BF3" s="28"/>
-      <c r="BG3" s="28"/>
-      <c r="BH3" s="28"/>
-      <c r="BI3" s="28"/>
-      <c r="BJ3" s="28"/>
-      <c r="BK3" s="28"/>
-      <c r="BL3" s="28"/>
-      <c r="BM3" s="28"/>
-      <c r="BN3" s="28"/>
-      <c r="BO3" s="28"/>
-      <c r="BP3" s="28"/>
-      <c r="BQ3" s="28"/>
-      <c r="BR3" s="28"/>
-      <c r="BS3" s="28"/>
-      <c r="BT3" s="28"/>
-      <c r="BU3" s="28"/>
-      <c r="BV3" s="28"/>
-      <c r="BW3" s="28"/>
-      <c r="BX3" s="28"/>
-      <c r="BY3" s="28"/>
-      <c r="BZ3" s="28"/>
-      <c r="CA3" s="30" t="s">
+      <c r="AW3" s="42"/>
+      <c r="AX3" s="42"/>
+      <c r="AY3" s="42"/>
+      <c r="AZ3" s="42"/>
+      <c r="BA3" s="42"/>
+      <c r="BB3" s="42"/>
+      <c r="BC3" s="42"/>
+      <c r="BD3" s="42"/>
+      <c r="BE3" s="42"/>
+      <c r="BF3" s="42"/>
+      <c r="BG3" s="42"/>
+      <c r="BH3" s="42"/>
+      <c r="BI3" s="42"/>
+      <c r="BJ3" s="42"/>
+      <c r="BK3" s="42"/>
+      <c r="BL3" s="42"/>
+      <c r="BM3" s="42"/>
+      <c r="BN3" s="42"/>
+      <c r="BO3" s="42"/>
+      <c r="BP3" s="42"/>
+      <c r="BQ3" s="42"/>
+      <c r="BR3" s="42"/>
+      <c r="BS3" s="42"/>
+      <c r="BT3" s="42"/>
+      <c r="BU3" s="42"/>
+      <c r="BV3" s="42"/>
+      <c r="BW3" s="42"/>
+      <c r="BX3" s="42"/>
+      <c r="BY3" s="42"/>
+      <c r="BZ3" s="42"/>
+      <c r="CA3" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="CB3" s="30"/>
-      <c r="CC3" s="30"/>
-      <c r="CD3" s="30"/>
-      <c r="CE3" s="30"/>
-      <c r="CF3" s="30"/>
-      <c r="CG3" s="30"/>
-      <c r="CH3" s="30"/>
-      <c r="CI3" s="30"/>
-      <c r="CJ3" s="30"/>
-      <c r="CK3" s="30"/>
-      <c r="CL3" s="30"/>
-      <c r="CM3" s="30"/>
-      <c r="CN3" s="30"/>
-      <c r="CO3" s="30"/>
-      <c r="CP3" s="30"/>
-      <c r="CQ3" s="30"/>
-      <c r="CR3" s="30"/>
-      <c r="CS3" s="30"/>
-      <c r="CT3" s="30"/>
-      <c r="CU3" s="30"/>
-      <c r="CV3" s="30"/>
-      <c r="CW3" s="30"/>
-      <c r="CX3" s="30"/>
-    </row>
-    <row r="4" spans="1:102">
-      <c r="A4" s="29"/>
-      <c r="B4" s="28" t="s">
+      <c r="CB3" s="45"/>
+      <c r="CC3" s="45"/>
+      <c r="CD3" s="45"/>
+      <c r="CE3" s="45"/>
+      <c r="CF3" s="45"/>
+      <c r="CG3" s="45"/>
+      <c r="CH3" s="45"/>
+      <c r="CI3" s="45"/>
+      <c r="CJ3" s="45"/>
+      <c r="CK3" s="45"/>
+      <c r="CL3" s="45"/>
+      <c r="CM3" s="45"/>
+      <c r="CN3" s="45"/>
+      <c r="CO3" s="45"/>
+      <c r="CP3" s="45"/>
+      <c r="CQ3" s="45"/>
+      <c r="CR3" s="45"/>
+      <c r="CS3" s="45"/>
+      <c r="CT3" s="45"/>
+      <c r="CU3" s="45"/>
+      <c r="CV3" s="45"/>
+      <c r="CW3" s="45"/>
+      <c r="CX3" s="45"/>
+    </row>
+    <row r="4" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A4" s="44"/>
+      <c r="B4" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="28"/>
+      <c r="C4" s="42"/>
       <c r="D4" t="s">
         <v>14</v>
       </c>
@@ -1449,12 +1524,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:102">
-      <c r="A5" s="29"/>
-      <c r="B5" s="28" t="s">
+    <row r="5" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A5" s="44"/>
+      <c r="B5" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="28"/>
+      <c r="C5" s="42"/>
       <c r="E5">
         <v>19</v>
       </c>
@@ -1844,13 +1919,13 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:102">
-      <c r="A6" s="29"/>
-      <c r="B6" s="28" t="s">
+    <row r="6" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A6" s="44"/>
+      <c r="B6" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="28"/>
-      <c r="D6" s="32"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="43"/>
       <c r="E6" s="6"/>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
@@ -1865,13 +1940,13 @@
       <c r="P6" s="7"/>
       <c r="Q6" s="8"/>
     </row>
-    <row r="7" spans="1:102">
-      <c r="A7" s="29"/>
-      <c r="B7" s="28" t="s">
+    <row r="7" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A7" s="44"/>
+      <c r="B7" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
       <c r="Q7" s="20"/>
       <c r="R7" s="21"/>
       <c r="S7" s="12"/>
@@ -1882,13 +1957,13 @@
       <c r="X7" s="12"/>
       <c r="Y7" s="12"/>
     </row>
-    <row r="8" spans="1:102">
-      <c r="A8" s="29"/>
-      <c r="B8" s="28" t="s">
+    <row r="8" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A8" s="44"/>
+      <c r="B8" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
       <c r="Q8" s="18"/>
       <c r="R8" s="19"/>
       <c r="S8" s="19"/>
@@ -1905,13 +1980,13 @@
       <c r="AD8" s="25"/>
       <c r="AE8" s="26"/>
     </row>
-    <row r="9" spans="1:102">
-      <c r="A9" s="29"/>
-      <c r="B9" s="28" t="s">
+    <row r="9" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A9" s="44"/>
+      <c r="B9" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
       <c r="AC9" s="22"/>
       <c r="AD9" s="19"/>
       <c r="AE9" s="19"/>
@@ -1919,13 +1994,13 @@
       <c r="AG9" s="19"/>
       <c r="AH9" s="23"/>
     </row>
-    <row r="10" spans="1:102">
-      <c r="A10" s="29"/>
-      <c r="B10" s="28" t="s">
+    <row r="10" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A10" s="44"/>
+      <c r="B10" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
       <c r="S10" s="14"/>
       <c r="T10" s="15"/>
       <c r="U10" s="15"/>
@@ -1935,13 +2010,13 @@
       <c r="Y10" s="15"/>
       <c r="Z10" s="17"/>
     </row>
-    <row r="11" spans="1:102">
-      <c r="A11" s="29"/>
-      <c r="B11" s="28" t="s">
+    <row r="11" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A11" s="44"/>
+      <c r="B11" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
       <c r="Z11" s="14"/>
       <c r="AA11" s="15"/>
       <c r="AB11" s="15"/>
@@ -1951,191 +2026,178 @@
       <c r="AF11" s="15"/>
       <c r="AG11" s="16"/>
     </row>
-    <row r="12" spans="1:102">
-      <c r="A12" s="29"/>
-      <c r="B12" s="28" t="s">
+    <row r="12" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A12" s="44"/>
+      <c r="B12" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
       <c r="AF12" s="14"/>
-      <c r="AG12" s="33"/>
+      <c r="AG12" s="28"/>
       <c r="AH12" s="17"/>
     </row>
-    <row r="13" spans="1:102">
-      <c r="A13" s="29"/>
-      <c r="B13" s="28" t="s">
+    <row r="13" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="44"/>
+      <c r="B13" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
       <c r="AG13" s="14"/>
       <c r="AH13" s="15"/>
       <c r="AI13" s="16"/>
     </row>
-    <row r="14" spans="1:102">
-      <c r="A14" s="29"/>
-      <c r="B14" s="28" t="s">
+    <row r="14" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="44"/>
+      <c r="B14" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="AH14" s="34"/>
-      <c r="AI14" s="35"/>
-      <c r="AJ14" s="15"/>
-      <c r="AK14" s="15"/>
-      <c r="AL14" s="16"/>
-    </row>
-    <row r="15" spans="1:102">
-      <c r="A15" s="29"/>
-      <c r="B15" s="28" t="s">
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
+      <c r="AH14" s="29"/>
+      <c r="AI14" s="13"/>
+      <c r="AJ14" s="28"/>
+      <c r="AK14" s="28"/>
+      <c r="AL14" s="15"/>
+      <c r="AM14" s="15"/>
+      <c r="AN14" s="17"/>
+    </row>
+    <row r="15" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="44"/>
+      <c r="B15" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="AH15" s="11"/>
-      <c r="AI15" s="11"/>
-      <c r="AJ15" s="11"/>
-      <c r="AK15" s="11"/>
-      <c r="AL15" s="11"/>
-      <c r="AM15" s="11"/>
-    </row>
-    <row r="16" spans="1:102">
-      <c r="A16" s="29"/>
-      <c r="B16" s="28" t="s">
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
+      <c r="AH15" s="30"/>
+      <c r="AI15" s="31"/>
+      <c r="AJ15" s="31"/>
+      <c r="AK15" s="31"/>
+      <c r="AL15" s="31"/>
+      <c r="AM15" s="32"/>
+    </row>
+    <row r="16" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="44"/>
+      <c r="B16" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="AK16" s="11"/>
-      <c r="AL16" s="11"/>
-      <c r="AM16" s="11"/>
-      <c r="AN16" s="11"/>
-      <c r="AO16" s="11"/>
-    </row>
-    <row r="17" spans="1:102">
-      <c r="A17" s="29"/>
-      <c r="B17" s="28" t="s">
+      <c r="C16" s="42"/>
+      <c r="D16" s="42"/>
+      <c r="AT16" s="33"/>
+      <c r="AU16" s="35"/>
+      <c r="AV16" s="35"/>
+      <c r="AW16" s="35"/>
+      <c r="AX16" s="35"/>
+      <c r="AY16" s="34"/>
+    </row>
+    <row r="17" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="44"/>
+      <c r="B17" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="AL17" s="13"/>
-      <c r="AM17" s="13"/>
-      <c r="AN17" s="13"/>
-      <c r="AO17" s="13"/>
-      <c r="AP17" s="13"/>
-    </row>
-    <row r="18" spans="1:102">
-      <c r="A18" s="29"/>
-      <c r="B18" s="28" t="s">
+      <c r="C17" s="42"/>
+      <c r="D17" s="42"/>
+      <c r="AU17" s="33"/>
+      <c r="AV17" s="35"/>
+      <c r="AW17" s="35"/>
+      <c r="AX17" s="35"/>
+      <c r="AY17" s="35"/>
+      <c r="AZ17" s="35"/>
+      <c r="BA17" s="34"/>
+    </row>
+    <row r="18" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="44"/>
+      <c r="B18" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="AN18" s="11"/>
-      <c r="AO18" s="11"/>
-      <c r="AP18" s="11"/>
-      <c r="AQ18" s="11"/>
-      <c r="AR18" s="11"/>
-      <c r="AS18" s="11"/>
-    </row>
-    <row r="19" spans="1:102">
-      <c r="A19" s="29"/>
-      <c r="B19" s="28" t="s">
+      <c r="C18" s="42"/>
+      <c r="D18" s="42"/>
+      <c r="BB18" s="14"/>
+      <c r="BC18" s="15"/>
+      <c r="BD18" s="15"/>
+      <c r="BE18" s="15"/>
+      <c r="BF18" s="15"/>
+      <c r="BG18" s="15"/>
+      <c r="BH18" s="16"/>
+    </row>
+    <row r="19" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="44"/>
+      <c r="B19" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="AQ19" s="11"/>
-      <c r="AR19" s="11"/>
-      <c r="AS19" s="11"/>
-      <c r="AT19" s="11"/>
-      <c r="AU19" s="11"/>
-      <c r="AV19" s="11"/>
-    </row>
-    <row r="20" spans="1:102">
-      <c r="A20" s="29"/>
-      <c r="B20" s="28" t="s">
+      <c r="C19" s="42"/>
+      <c r="D19" s="42"/>
+      <c r="BH19" s="33"/>
+      <c r="BI19" s="35"/>
+      <c r="BJ19" s="35"/>
+      <c r="BK19" s="35"/>
+      <c r="BL19" s="41"/>
+    </row>
+    <row r="20" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A20" s="44"/>
+      <c r="B20" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="AQ20" s="13"/>
-      <c r="AR20" s="13"/>
-      <c r="AS20" s="13"/>
-      <c r="AT20" s="13"/>
-      <c r="AU20" s="13"/>
-      <c r="AV20" s="13"/>
-      <c r="AW20" s="13"/>
-      <c r="AX20" s="13"/>
-    </row>
-    <row r="21" spans="1:102">
-      <c r="A21" s="29"/>
-      <c r="B21" s="28" t="s">
+      <c r="C20" s="42"/>
+      <c r="D20" s="42"/>
+      <c r="BH20" s="37"/>
+      <c r="BI20" s="38"/>
+      <c r="BJ20" s="38"/>
+      <c r="BK20" s="38"/>
+      <c r="BL20" s="39"/>
+    </row>
+    <row r="21" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A21" s="44"/>
+      <c r="B21" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="AV21" s="11"/>
-      <c r="AW21" s="11"/>
-      <c r="AX21" s="11"/>
-      <c r="AY21" s="11"/>
-      <c r="AZ21" s="11"/>
-      <c r="BA21" s="11"/>
-      <c r="BB21" s="11"/>
-      <c r="BC21" s="11"/>
-      <c r="BD21" s="11"/>
-    </row>
-    <row r="22" spans="1:102">
-      <c r="A22" s="29"/>
-      <c r="B22" s="28" t="s">
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
+      <c r="BM21" s="11"/>
+      <c r="BN21" s="11"/>
+      <c r="BO21" s="11"/>
+      <c r="BP21" s="11"/>
+    </row>
+    <row r="22" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A22" s="44"/>
+      <c r="B22" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="BB22" s="27"/>
-      <c r="BC22" s="27"/>
-      <c r="BD22" s="27"/>
-      <c r="BE22" s="27"/>
-      <c r="BF22" s="27"/>
-      <c r="BG22" s="27"/>
-      <c r="BH22" s="27"/>
-      <c r="BI22" s="27"/>
-      <c r="BJ22" s="27"/>
-    </row>
-    <row r="23" spans="1:102">
-      <c r="A23" s="29"/>
-      <c r="B23" s="28" t="s">
+      <c r="C22" s="42"/>
+      <c r="D22" s="42"/>
+      <c r="BQ22" s="11"/>
+      <c r="BR22" s="11"/>
+      <c r="BS22" s="11"/>
+      <c r="BT22" s="11"/>
+      <c r="BU22" s="11"/>
+      <c r="BV22" s="11"/>
+    </row>
+    <row r="23" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A23" s="44"/>
+      <c r="B23" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="BK23" s="27"/>
-      <c r="BL23" s="27"/>
-      <c r="BM23" s="27"/>
-      <c r="BN23" s="27"/>
-      <c r="BO23" s="27"/>
-      <c r="BP23" s="27"/>
-      <c r="BQ23" s="27"/>
-      <c r="BR23" s="27"/>
-      <c r="BS23" s="27"/>
-      <c r="BT23" s="27"/>
-      <c r="BU23" s="27"/>
-      <c r="BV23" s="27"/>
-      <c r="BW23" s="27"/>
-      <c r="BX23" s="27"/>
-      <c r="BY23" s="27"/>
-      <c r="BZ23" s="27"/>
-      <c r="CA23" s="27"/>
-    </row>
-    <row r="24" spans="1:102">
-      <c r="A24" s="29"/>
-      <c r="B24" s="28" t="s">
+      <c r="C23" s="42"/>
+      <c r="D23" s="42"/>
+      <c r="BM23" s="13"/>
+      <c r="BN23" s="13"/>
+      <c r="BO23" s="13"/>
+      <c r="BP23" s="13"/>
+      <c r="BQ23" s="13"/>
+      <c r="BR23" s="13"/>
+      <c r="BS23" s="13"/>
+      <c r="BT23" s="13"/>
+      <c r="BU23" s="13"/>
+      <c r="BV23" s="13"/>
+    </row>
+    <row r="24" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A24" s="44"/>
+      <c r="B24" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="28"/>
-      <c r="D24" s="28"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="42"/>
       <c r="BR24" s="27"/>
       <c r="BS24" s="27"/>
       <c r="BT24" s="27"/>
@@ -2153,302 +2215,199 @@
       <c r="CF24" s="27"/>
       <c r="CG24" s="27"/>
       <c r="CH24" s="27"/>
-      <c r="CI24" s="27"/>
-      <c r="CJ24" s="27"/>
-      <c r="CK24" s="27"/>
-      <c r="CL24" s="27"/>
-      <c r="CM24" s="27"/>
-      <c r="CN24" s="27"/>
-      <c r="CO24" s="27"/>
-      <c r="CP24" s="27"/>
-      <c r="CQ24" s="27"/>
-      <c r="CR24" s="27"/>
-      <c r="CS24" s="27"/>
-      <c r="CT24" s="27"/>
-      <c r="CU24" s="27"/>
-      <c r="CV24" s="27"/>
-      <c r="CW24" s="27"/>
-      <c r="CX24" s="27"/>
-    </row>
-    <row r="25" spans="1:102">
-      <c r="A25" s="29"/>
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-    </row>
-    <row r="26" spans="1:102">
-      <c r="A26" s="29"/>
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-    </row>
-    <row r="27" spans="1:102">
-      <c r="A27" s="29"/>
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-    </row>
-    <row r="28" spans="1:102">
-      <c r="A28" s="29"/>
-      <c r="B28" s="28" t="s">
+    </row>
+    <row r="25" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A25" s="44"/>
+      <c r="B25" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="AF28" s="13"/>
-      <c r="AG28" s="13"/>
-      <c r="AH28" s="13"/>
-      <c r="AI28" s="13"/>
-      <c r="AJ28" s="13"/>
-      <c r="AK28" s="13"/>
-      <c r="AL28" s="13"/>
-      <c r="AM28" s="13"/>
-      <c r="AN28" s="13"/>
-    </row>
-    <row r="29" spans="1:102">
-      <c r="A29" s="29"/>
-      <c r="B29" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="AK29" s="11"/>
-      <c r="AL29" s="11"/>
-      <c r="AM29" s="11"/>
-      <c r="AN29" s="11"/>
-      <c r="AO29" s="11"/>
-      <c r="AP29" s="11"/>
-      <c r="AQ29" s="11"/>
-      <c r="AR29" s="11"/>
-      <c r="AS29" s="11"/>
-      <c r="AT29" s="11"/>
-      <c r="AU29" s="11"/>
-      <c r="AV29" s="11"/>
-    </row>
-    <row r="30" spans="1:102">
-      <c r="A30" s="29"/>
-      <c r="B30" s="28" t="s">
-        <v>43</v>
-      </c>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="AF30" s="11"/>
-      <c r="AG30" s="11"/>
-      <c r="AH30" s="11"/>
-      <c r="AI30" s="11"/>
-      <c r="AJ30" s="11"/>
-      <c r="AK30" s="11"/>
-      <c r="AL30" s="11"/>
-      <c r="AM30" s="11"/>
-      <c r="AN30" s="11"/>
-      <c r="AO30" s="11"/>
-    </row>
-    <row r="31" spans="1:102">
-      <c r="A31" s="29"/>
-      <c r="B31" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28"/>
-      <c r="AV31" s="13"/>
-      <c r="AW31" s="13"/>
-      <c r="AX31" s="13"/>
-      <c r="AY31" s="13"/>
-      <c r="AZ31" s="13"/>
-      <c r="BA31" s="13"/>
-      <c r="BB31" s="13"/>
-      <c r="BC31" s="13"/>
-      <c r="BD31" s="13"/>
-      <c r="BE31" s="13"/>
-      <c r="BF31" s="13"/>
-    </row>
-    <row r="32" spans="1:102">
-      <c r="A32" s="29"/>
-      <c r="B32" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="AV32" s="11"/>
-      <c r="AW32" s="11"/>
-      <c r="AX32" s="11"/>
-      <c r="AY32" s="11"/>
-      <c r="AZ32" s="11"/>
-      <c r="BA32" s="11"/>
-      <c r="BB32" s="11"/>
-      <c r="BC32" s="11"/>
-      <c r="BD32" s="11"/>
-      <c r="BE32" s="11"/>
-      <c r="BF32" s="11"/>
-    </row>
-    <row r="33" spans="1:102">
-      <c r="A33" s="29"/>
-      <c r="B33" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="C33" s="28"/>
-      <c r="D33" s="28"/>
-      <c r="AN33" s="13"/>
-      <c r="AO33" s="13"/>
-      <c r="AP33" s="13"/>
-      <c r="AQ33" s="13"/>
-      <c r="AR33" s="13"/>
-      <c r="AS33" s="13"/>
-      <c r="AT33" s="13"/>
-      <c r="AU33" s="13"/>
-      <c r="AV33" s="13"/>
-      <c r="AW33" s="13"/>
-      <c r="AX33" s="13"/>
-      <c r="AY33" s="13"/>
-      <c r="AZ33" s="13"/>
-      <c r="BA33" s="13"/>
-      <c r="BB33" s="13"/>
-    </row>
-    <row r="34" spans="1:102">
-      <c r="A34" s="29"/>
-      <c r="B34" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="C34" s="28"/>
-      <c r="D34" s="28"/>
-      <c r="BG34" s="27"/>
-      <c r="BH34" s="27"/>
-      <c r="BI34" s="27"/>
-      <c r="BJ34" s="27"/>
-      <c r="BK34" s="27"/>
-      <c r="BL34" s="27"/>
-      <c r="BM34" s="27"/>
-      <c r="BN34" s="27"/>
-      <c r="BO34" s="27"/>
-      <c r="BP34" s="27"/>
-      <c r="BQ34" s="27"/>
-      <c r="BR34" s="27"/>
-      <c r="BS34" s="27"/>
-      <c r="BT34" s="27"/>
-      <c r="BU34" s="27"/>
-      <c r="BV34" s="27"/>
-      <c r="BW34" s="27"/>
-      <c r="BX34" s="27"/>
-      <c r="BY34" s="27"/>
-      <c r="BZ34" s="27"/>
-      <c r="CA34" s="27"/>
-      <c r="CB34" s="27"/>
-      <c r="CC34" s="27"/>
-      <c r="CD34" s="27"/>
-      <c r="CE34" s="27"/>
-      <c r="CF34" s="27"/>
-      <c r="CG34" s="27"/>
-      <c r="CH34" s="27"/>
-      <c r="CI34" s="27"/>
-      <c r="CJ34" s="27"/>
-      <c r="CK34" s="27"/>
-      <c r="CL34" s="27"/>
-      <c r="CM34" s="27"/>
-      <c r="CN34" s="27"/>
-      <c r="CO34" s="27"/>
-      <c r="CP34" s="27"/>
-      <c r="CQ34" s="27"/>
-      <c r="CR34" s="27"/>
-      <c r="CS34" s="27"/>
-      <c r="CT34" s="27"/>
-      <c r="CU34" s="27"/>
-      <c r="CV34" s="27"/>
-      <c r="CW34" s="27"/>
-      <c r="CX34" s="27"/>
-    </row>
-    <row r="35" spans="1:102">
-      <c r="A35" s="29"/>
-      <c r="B35" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C35" s="28"/>
-      <c r="D35" s="28"/>
-      <c r="BG35" s="27"/>
-      <c r="BH35" s="27"/>
-      <c r="BI35" s="27"/>
-      <c r="BJ35" s="27"/>
-      <c r="BK35" s="27"/>
-      <c r="BL35" s="27"/>
-      <c r="BM35" s="27"/>
-      <c r="BN35" s="27"/>
-      <c r="BO35" s="27"/>
-    </row>
-    <row r="36" spans="1:102">
-      <c r="A36" s="29"/>
-      <c r="B36" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="C36" s="28"/>
-      <c r="D36" s="28"/>
-      <c r="BP36" s="27"/>
-      <c r="BQ36" s="27"/>
-      <c r="BR36" s="27"/>
-      <c r="BS36" s="27"/>
-      <c r="BT36" s="27"/>
-      <c r="BU36" s="27"/>
-      <c r="BV36" s="27"/>
-      <c r="BW36" s="27"/>
-      <c r="BX36" s="27"/>
-      <c r="BY36" s="27"/>
-      <c r="BZ36" s="27"/>
-      <c r="CA36" s="27"/>
-      <c r="CB36" s="27"/>
-      <c r="CC36" s="27"/>
-      <c r="CD36" s="27"/>
-      <c r="CE36" s="27"/>
-      <c r="CF36" s="27"/>
-      <c r="CG36" s="27"/>
-      <c r="CH36" s="27"/>
-      <c r="CI36" s="27"/>
-      <c r="CJ36" s="27"/>
-      <c r="CK36" s="27"/>
-      <c r="CL36" s="27"/>
-      <c r="CM36" s="27"/>
-      <c r="CN36" s="27"/>
-      <c r="CO36" s="27"/>
-      <c r="CP36" s="27"/>
-      <c r="CQ36" s="27"/>
-      <c r="CR36" s="27"/>
-      <c r="CS36" s="27"/>
-      <c r="CT36" s="27"/>
-      <c r="CU36" s="27"/>
-      <c r="CV36" s="27"/>
-      <c r="CW36" s="27"/>
-      <c r="CX36" s="27"/>
-    </row>
-    <row r="37" spans="1:102">
-      <c r="A37" s="29"/>
-    </row>
-    <row r="38" spans="1:102">
-      <c r="A38" s="29"/>
-    </row>
-    <row r="39" spans="1:102">
-      <c r="A39" s="29"/>
-    </row>
-    <row r="40" spans="1:102">
-      <c r="A40" s="29"/>
-    </row>
-    <row r="41" spans="1:102">
-      <c r="A41" s="29"/>
-    </row>
-    <row r="42" spans="1:102">
-      <c r="A42" s="29"/>
-    </row>
-    <row r="43" spans="1:102">
-      <c r="A43" s="29"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="42"/>
+      <c r="BY25" s="27"/>
+      <c r="BZ25" s="27"/>
+      <c r="CA25" s="27"/>
+      <c r="CB25" s="27"/>
+      <c r="CC25" s="27"/>
+      <c r="CD25" s="27"/>
+      <c r="CE25" s="27"/>
+      <c r="CF25" s="27"/>
+      <c r="CG25" s="27"/>
+      <c r="CH25" s="27"/>
+      <c r="CI25" s="27"/>
+      <c r="CJ25" s="27"/>
+      <c r="CK25" s="27"/>
+      <c r="CL25" s="27"/>
+      <c r="CM25" s="27"/>
+      <c r="CN25" s="27"/>
+      <c r="CO25" s="27"/>
+      <c r="CP25" s="27"/>
+      <c r="CQ25" s="27"/>
+      <c r="CR25" s="27"/>
+      <c r="CS25" s="27"/>
+      <c r="CT25" s="27"/>
+      <c r="CU25" s="27"/>
+      <c r="CV25" s="27"/>
+      <c r="CW25" s="27"/>
+      <c r="CX25" s="27"/>
+    </row>
+    <row r="26" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A26" s="44"/>
+      <c r="B26" s="42"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="42"/>
+    </row>
+    <row r="27" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A27" s="44"/>
+      <c r="B27" s="42"/>
+      <c r="C27" s="42"/>
+      <c r="D27" s="42"/>
+    </row>
+    <row r="28" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A28" s="44"/>
+      <c r="B28" s="42"/>
+      <c r="C28" s="42"/>
+      <c r="D28" s="42"/>
+    </row>
+    <row r="29" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A29" s="44"/>
+    </row>
+    <row r="30" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A30" s="44"/>
+      <c r="AS30" s="40"/>
+    </row>
+    <row r="31" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A31" s="44"/>
+    </row>
+    <row r="32" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A32" s="44"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="44"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="44"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" s="44"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="36"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" s="36"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" s="36"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" s="36"/>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" s="36"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" s="36"/>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" s="36"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" s="36"/>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" s="36"/>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" s="36"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" s="36"/>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" s="36"/>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A48" s="36"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" s="36"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" s="36"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A51" s="36"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A52" s="36"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A53" s="36"/>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A54" s="36"/>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A55" s="36"/>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A56" s="36"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A57" s="36"/>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A58" s="36"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A59" s="36"/>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A60" s="36"/>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A61" s="36"/>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A62" s="36"/>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A63" s="36"/>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A64" s="36"/>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A65" s="36"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A66" s="36"/>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A67" s="36"/>
     </row>
   </sheetData>
-  <mergeCells count="44">
-    <mergeCell ref="B27:D27"/>
+  <mergeCells count="36">
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B20:D20"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B21:D21"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="K2:M2"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
     <mergeCell ref="P2:R2"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="A1:CX1"/>
@@ -2459,30 +2418,12 @@
     <mergeCell ref="AV3:BZ3"/>
     <mergeCell ref="R3:AU3"/>
     <mergeCell ref="E3:Q3"/>
-    <mergeCell ref="A2:A43"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="A2:A35"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B36:D36"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B22:D22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
mise à jour du Gantt
</commit_message>
<xml_diff>
--- a/Gantt Mastermind.xlsx
+++ b/Gantt Mastermind.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dimitricourtoisrozelot/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dimitricourtoisrozelot/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D27BDB2-7814-1C42-A224-D3B8FD851E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7755690-B610-C942-ACD3-0EB3E2CEC02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1120" yWindow="740" windowWidth="28280" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="48">
   <si>
     <t>Mastermind</t>
   </si>
@@ -172,19 +172,31 @@
     <t>améliorer l'affichage des lignes validées</t>
   </si>
   <si>
-    <t>ajout d'option(abandonner,,,)</t>
+    <t>ajout niveau de difficulté</t>
+  </si>
+  <si>
+    <t>améliorer ecran de victoire (nb tentative+option quitter)</t>
+  </si>
+  <si>
+    <t>ajouter explication des règles</t>
+  </si>
+  <si>
+    <t>ajout d'effet sonore</t>
+  </si>
+  <si>
+    <t>amélioration de la manière de lancer</t>
   </si>
   <si>
     <t>Améliorier l'esthétique</t>
   </si>
   <si>
-    <t>ajouter un bouton abandonner</t>
-  </si>
-  <si>
-    <t>ajout du niveau medium et hard</t>
-  </si>
-  <si>
-    <t>améliorer ecran de victoire (nb tentative+option quitter)</t>
+    <t>ajouter des boutons quitter</t>
+  </si>
+  <si>
+    <t>ajout d'une option pour limiter le nombre d'essai</t>
+  </si>
+  <si>
+    <t>Curseur de sourie de la couleur selectionée</t>
   </si>
 </sst>
 </file>
@@ -283,7 +295,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -490,11 +502,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF00B050"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF00B050"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF00B050"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF00B050"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -561,6 +602,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -579,7 +622,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -946,142 +991,142 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="42"/>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
-      <c r="S1" s="42"/>
-      <c r="T1" s="42"/>
-      <c r="U1" s="42"/>
-      <c r="V1" s="42"/>
-      <c r="W1" s="42"/>
-      <c r="X1" s="42"/>
-      <c r="Y1" s="42"/>
-      <c r="Z1" s="42"/>
-      <c r="AA1" s="42"/>
-      <c r="AB1" s="42"/>
-      <c r="AC1" s="42"/>
-      <c r="AD1" s="42"/>
-      <c r="AE1" s="42"/>
-      <c r="AF1" s="42"/>
-      <c r="AG1" s="42"/>
-      <c r="AH1" s="42"/>
-      <c r="AI1" s="42"/>
-      <c r="AJ1" s="42"/>
-      <c r="AK1" s="42"/>
-      <c r="AL1" s="42"/>
-      <c r="AM1" s="42"/>
-      <c r="AN1" s="42"/>
-      <c r="AO1" s="42"/>
-      <c r="AP1" s="42"/>
-      <c r="AQ1" s="42"/>
-      <c r="AR1" s="42"/>
-      <c r="AS1" s="42"/>
-      <c r="AT1" s="42"/>
-      <c r="AU1" s="42"/>
-      <c r="AV1" s="42"/>
-      <c r="AW1" s="42"/>
-      <c r="AX1" s="42"/>
-      <c r="AY1" s="42"/>
-      <c r="AZ1" s="42"/>
-      <c r="BA1" s="42"/>
-      <c r="BB1" s="42"/>
-      <c r="BC1" s="42"/>
-      <c r="BD1" s="42"/>
-      <c r="BE1" s="42"/>
-      <c r="BF1" s="42"/>
-      <c r="BG1" s="42"/>
-      <c r="BH1" s="42"/>
-      <c r="BI1" s="42"/>
-      <c r="BJ1" s="42"/>
-      <c r="BK1" s="42"/>
-      <c r="BL1" s="42"/>
-      <c r="BM1" s="42"/>
-      <c r="BN1" s="42"/>
-      <c r="BO1" s="42"/>
-      <c r="BP1" s="42"/>
-      <c r="BQ1" s="42"/>
-      <c r="BR1" s="42"/>
-      <c r="BS1" s="42"/>
-      <c r="BT1" s="42"/>
-      <c r="BU1" s="42"/>
-      <c r="BV1" s="42"/>
-      <c r="BW1" s="42"/>
-      <c r="BX1" s="42"/>
-      <c r="BY1" s="42"/>
-      <c r="BZ1" s="42"/>
-      <c r="CA1" s="42"/>
-      <c r="CB1" s="42"/>
-      <c r="CC1" s="42"/>
-      <c r="CD1" s="42"/>
-      <c r="CE1" s="42"/>
-      <c r="CF1" s="42"/>
-      <c r="CG1" s="42"/>
-      <c r="CH1" s="42"/>
-      <c r="CI1" s="42"/>
-      <c r="CJ1" s="42"/>
-      <c r="CK1" s="42"/>
-      <c r="CL1" s="42"/>
-      <c r="CM1" s="42"/>
-      <c r="CN1" s="42"/>
-      <c r="CO1" s="42"/>
-      <c r="CP1" s="42"/>
-      <c r="CQ1" s="42"/>
-      <c r="CR1" s="42"/>
-      <c r="CS1" s="42"/>
-      <c r="CT1" s="42"/>
-      <c r="CU1" s="42"/>
-      <c r="CV1" s="42"/>
-      <c r="CW1" s="42"/>
-      <c r="CX1" s="42"/>
+      <c r="A1" s="44"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
+      <c r="P1" s="44"/>
+      <c r="Q1" s="44"/>
+      <c r="R1" s="44"/>
+      <c r="S1" s="44"/>
+      <c r="T1" s="44"/>
+      <c r="U1" s="44"/>
+      <c r="V1" s="44"/>
+      <c r="W1" s="44"/>
+      <c r="X1" s="44"/>
+      <c r="Y1" s="44"/>
+      <c r="Z1" s="44"/>
+      <c r="AA1" s="44"/>
+      <c r="AB1" s="44"/>
+      <c r="AC1" s="44"/>
+      <c r="AD1" s="44"/>
+      <c r="AE1" s="44"/>
+      <c r="AF1" s="44"/>
+      <c r="AG1" s="44"/>
+      <c r="AH1" s="44"/>
+      <c r="AI1" s="44"/>
+      <c r="AJ1" s="44"/>
+      <c r="AK1" s="44"/>
+      <c r="AL1" s="44"/>
+      <c r="AM1" s="44"/>
+      <c r="AN1" s="44"/>
+      <c r="AO1" s="44"/>
+      <c r="AP1" s="44"/>
+      <c r="AQ1" s="44"/>
+      <c r="AR1" s="44"/>
+      <c r="AS1" s="44"/>
+      <c r="AT1" s="44"/>
+      <c r="AU1" s="44"/>
+      <c r="AV1" s="44"/>
+      <c r="AW1" s="44"/>
+      <c r="AX1" s="44"/>
+      <c r="AY1" s="44"/>
+      <c r="AZ1" s="44"/>
+      <c r="BA1" s="44"/>
+      <c r="BB1" s="44"/>
+      <c r="BC1" s="44"/>
+      <c r="BD1" s="44"/>
+      <c r="BE1" s="44"/>
+      <c r="BF1" s="44"/>
+      <c r="BG1" s="44"/>
+      <c r="BH1" s="44"/>
+      <c r="BI1" s="44"/>
+      <c r="BJ1" s="44"/>
+      <c r="BK1" s="44"/>
+      <c r="BL1" s="44"/>
+      <c r="BM1" s="44"/>
+      <c r="BN1" s="44"/>
+      <c r="BO1" s="44"/>
+      <c r="BP1" s="44"/>
+      <c r="BQ1" s="44"/>
+      <c r="BR1" s="44"/>
+      <c r="BS1" s="44"/>
+      <c r="BT1" s="44"/>
+      <c r="BU1" s="44"/>
+      <c r="BV1" s="44"/>
+      <c r="BW1" s="44"/>
+      <c r="BX1" s="44"/>
+      <c r="BY1" s="44"/>
+      <c r="BZ1" s="44"/>
+      <c r="CA1" s="44"/>
+      <c r="CB1" s="44"/>
+      <c r="CC1" s="44"/>
+      <c r="CD1" s="44"/>
+      <c r="CE1" s="44"/>
+      <c r="CF1" s="44"/>
+      <c r="CG1" s="44"/>
+      <c r="CH1" s="44"/>
+      <c r="CI1" s="44"/>
+      <c r="CJ1" s="44"/>
+      <c r="CK1" s="44"/>
+      <c r="CL1" s="44"/>
+      <c r="CM1" s="44"/>
+      <c r="CN1" s="44"/>
+      <c r="CO1" s="44"/>
+      <c r="CP1" s="44"/>
+      <c r="CQ1" s="44"/>
+      <c r="CR1" s="44"/>
+      <c r="CS1" s="44"/>
+      <c r="CT1" s="44"/>
+      <c r="CU1" s="44"/>
+      <c r="CV1" s="44"/>
+      <c r="CW1" s="44"/>
+      <c r="CX1" s="44"/>
     </row>
     <row r="2" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42"/>
-      <c r="B2" s="38" t="s">
+      <c r="A2" s="44"/>
+      <c r="B2" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
       <c r="I2" s="1"/>
       <c r="J2" s="4"/>
-      <c r="K2" s="40" t="s">
+      <c r="K2" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="38"/>
-      <c r="M2" s="38"/>
+      <c r="L2" s="40"/>
+      <c r="M2" s="40"/>
       <c r="O2" s="2"/>
-      <c r="P2" s="38" t="s">
+      <c r="P2" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="Q2" s="38"/>
-      <c r="R2" s="38"/>
+      <c r="Q2" s="40"/>
+      <c r="R2" s="40"/>
       <c r="S2" s="1"/>
       <c r="T2" s="5"/>
-      <c r="U2" s="38" t="s">
+      <c r="U2" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="V2" s="38"/>
-      <c r="W2" s="38"/>
+      <c r="V2" s="40"/>
+      <c r="W2" s="40"/>
       <c r="X2" s="1"/>
       <c r="Y2" s="3"/>
       <c r="Z2" t="s">
@@ -1089,7 +1134,7 @@
       </c>
     </row>
     <row r="3" spans="1:102" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="42"/>
+      <c r="A3" s="44"/>
       <c r="B3" s="10" t="s">
         <v>6</v>
       </c>
@@ -1099,119 +1144,119 @@
       <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="E3" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="38"/>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="38"/>
-      <c r="J3" s="38"/>
-      <c r="K3" s="38"/>
-      <c r="L3" s="38"/>
-      <c r="M3" s="38"/>
-      <c r="N3" s="38"/>
-      <c r="O3" s="38"/>
-      <c r="P3" s="38"/>
-      <c r="Q3" s="38"/>
-      <c r="R3" s="38" t="s">
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="40"/>
+      <c r="N3" s="40"/>
+      <c r="O3" s="40"/>
+      <c r="P3" s="40"/>
+      <c r="Q3" s="40"/>
+      <c r="R3" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="S3" s="38"/>
-      <c r="T3" s="38"/>
-      <c r="U3" s="38"/>
-      <c r="V3" s="38"/>
-      <c r="W3" s="38"/>
-      <c r="X3" s="38"/>
-      <c r="Y3" s="38"/>
-      <c r="Z3" s="38"/>
-      <c r="AA3" s="38"/>
-      <c r="AB3" s="38"/>
-      <c r="AC3" s="38"/>
-      <c r="AD3" s="38"/>
-      <c r="AE3" s="38"/>
-      <c r="AF3" s="38"/>
-      <c r="AG3" s="38"/>
-      <c r="AH3" s="38"/>
-      <c r="AI3" s="38"/>
-      <c r="AJ3" s="38"/>
-      <c r="AK3" s="38"/>
-      <c r="AL3" s="38"/>
-      <c r="AM3" s="38"/>
-      <c r="AN3" s="38"/>
-      <c r="AO3" s="38"/>
-      <c r="AP3" s="38"/>
-      <c r="AQ3" s="38"/>
-      <c r="AR3" s="38"/>
-      <c r="AS3" s="38"/>
-      <c r="AT3" s="38"/>
-      <c r="AU3" s="38"/>
-      <c r="AV3" s="38" t="s">
+      <c r="S3" s="40"/>
+      <c r="T3" s="40"/>
+      <c r="U3" s="40"/>
+      <c r="V3" s="40"/>
+      <c r="W3" s="40"/>
+      <c r="X3" s="40"/>
+      <c r="Y3" s="40"/>
+      <c r="Z3" s="40"/>
+      <c r="AA3" s="40"/>
+      <c r="AB3" s="40"/>
+      <c r="AC3" s="40"/>
+      <c r="AD3" s="40"/>
+      <c r="AE3" s="40"/>
+      <c r="AF3" s="40"/>
+      <c r="AG3" s="40"/>
+      <c r="AH3" s="40"/>
+      <c r="AI3" s="40"/>
+      <c r="AJ3" s="40"/>
+      <c r="AK3" s="40"/>
+      <c r="AL3" s="40"/>
+      <c r="AM3" s="40"/>
+      <c r="AN3" s="40"/>
+      <c r="AO3" s="40"/>
+      <c r="AP3" s="40"/>
+      <c r="AQ3" s="40"/>
+      <c r="AR3" s="40"/>
+      <c r="AS3" s="40"/>
+      <c r="AT3" s="40"/>
+      <c r="AU3" s="40"/>
+      <c r="AV3" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="AW3" s="38"/>
-      <c r="AX3" s="38"/>
-      <c r="AY3" s="38"/>
-      <c r="AZ3" s="38"/>
-      <c r="BA3" s="38"/>
-      <c r="BB3" s="38"/>
-      <c r="BC3" s="38"/>
-      <c r="BD3" s="38"/>
-      <c r="BE3" s="38"/>
-      <c r="BF3" s="38"/>
-      <c r="BG3" s="38"/>
-      <c r="BH3" s="38"/>
-      <c r="BI3" s="38"/>
-      <c r="BJ3" s="38"/>
-      <c r="BK3" s="38"/>
-      <c r="BL3" s="38"/>
-      <c r="BM3" s="38"/>
-      <c r="BN3" s="38"/>
-      <c r="BO3" s="38"/>
-      <c r="BP3" s="38"/>
-      <c r="BQ3" s="38"/>
-      <c r="BR3" s="38"/>
-      <c r="BS3" s="38"/>
-      <c r="BT3" s="38"/>
-      <c r="BU3" s="38"/>
-      <c r="BV3" s="38"/>
-      <c r="BW3" s="38"/>
-      <c r="BX3" s="38"/>
-      <c r="BY3" s="38"/>
-      <c r="BZ3" s="38"/>
-      <c r="CA3" s="43" t="s">
+      <c r="AW3" s="40"/>
+      <c r="AX3" s="40"/>
+      <c r="AY3" s="40"/>
+      <c r="AZ3" s="40"/>
+      <c r="BA3" s="40"/>
+      <c r="BB3" s="40"/>
+      <c r="BC3" s="40"/>
+      <c r="BD3" s="40"/>
+      <c r="BE3" s="40"/>
+      <c r="BF3" s="40"/>
+      <c r="BG3" s="40"/>
+      <c r="BH3" s="40"/>
+      <c r="BI3" s="40"/>
+      <c r="BJ3" s="40"/>
+      <c r="BK3" s="40"/>
+      <c r="BL3" s="40"/>
+      <c r="BM3" s="40"/>
+      <c r="BN3" s="40"/>
+      <c r="BO3" s="40"/>
+      <c r="BP3" s="40"/>
+      <c r="BQ3" s="40"/>
+      <c r="BR3" s="40"/>
+      <c r="BS3" s="40"/>
+      <c r="BT3" s="40"/>
+      <c r="BU3" s="40"/>
+      <c r="BV3" s="40"/>
+      <c r="BW3" s="40"/>
+      <c r="BX3" s="40"/>
+      <c r="BY3" s="40"/>
+      <c r="BZ3" s="40"/>
+      <c r="CA3" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="CB3" s="43"/>
-      <c r="CC3" s="43"/>
-      <c r="CD3" s="43"/>
-      <c r="CE3" s="43"/>
-      <c r="CF3" s="43"/>
-      <c r="CG3" s="43"/>
-      <c r="CH3" s="43"/>
-      <c r="CI3" s="43"/>
-      <c r="CJ3" s="43"/>
-      <c r="CK3" s="43"/>
-      <c r="CL3" s="43"/>
-      <c r="CM3" s="43"/>
-      <c r="CN3" s="43"/>
-      <c r="CO3" s="43"/>
-      <c r="CP3" s="43"/>
-      <c r="CQ3" s="43"/>
-      <c r="CR3" s="43"/>
-      <c r="CS3" s="43"/>
-      <c r="CT3" s="43"/>
-      <c r="CU3" s="43"/>
-      <c r="CV3" s="43"/>
-      <c r="CW3" s="43"/>
-      <c r="CX3" s="43"/>
+      <c r="CB3" s="45"/>
+      <c r="CC3" s="45"/>
+      <c r="CD3" s="45"/>
+      <c r="CE3" s="45"/>
+      <c r="CF3" s="45"/>
+      <c r="CG3" s="45"/>
+      <c r="CH3" s="45"/>
+      <c r="CI3" s="45"/>
+      <c r="CJ3" s="45"/>
+      <c r="CK3" s="45"/>
+      <c r="CL3" s="45"/>
+      <c r="CM3" s="45"/>
+      <c r="CN3" s="45"/>
+      <c r="CO3" s="45"/>
+      <c r="CP3" s="45"/>
+      <c r="CQ3" s="45"/>
+      <c r="CR3" s="45"/>
+      <c r="CS3" s="45"/>
+      <c r="CT3" s="45"/>
+      <c r="CU3" s="45"/>
+      <c r="CV3" s="45"/>
+      <c r="CW3" s="45"/>
+      <c r="CX3" s="45"/>
     </row>
     <row r="4" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A4" s="42"/>
-      <c r="B4" s="38" t="s">
+      <c r="A4" s="44"/>
+      <c r="B4" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="38"/>
+      <c r="C4" s="40"/>
       <c r="D4" t="s">
         <v>14</v>
       </c>
@@ -1511,11 +1556,11 @@
       </c>
     </row>
     <row r="5" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A5" s="42"/>
-      <c r="B5" s="38" t="s">
+      <c r="A5" s="44"/>
+      <c r="B5" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="38"/>
+      <c r="C5" s="40"/>
       <c r="E5">
         <v>19</v>
       </c>
@@ -1906,12 +1951,12 @@
       </c>
     </row>
     <row r="6" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A6" s="42"/>
-      <c r="B6" s="38" t="s">
+      <c r="A6" s="44"/>
+      <c r="B6" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="38"/>
-      <c r="D6" s="41"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="43"/>
       <c r="E6" s="6"/>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
@@ -1927,12 +1972,12 @@
       <c r="Q6" s="8"/>
     </row>
     <row r="7" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A7" s="42"/>
-      <c r="B7" s="38" t="s">
+      <c r="A7" s="44"/>
+      <c r="B7" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="38"/>
-      <c r="D7" s="38"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
       <c r="Q7" s="20"/>
       <c r="R7" s="21"/>
       <c r="S7" s="12"/>
@@ -1944,12 +1989,12 @@
       <c r="Y7" s="12"/>
     </row>
     <row r="8" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A8" s="42"/>
-      <c r="B8" s="38" t="s">
+      <c r="A8" s="44"/>
+      <c r="B8" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
       <c r="Q8" s="18"/>
       <c r="R8" s="19"/>
       <c r="S8" s="19"/>
@@ -1967,12 +2012,12 @@
       <c r="AE8" s="26"/>
     </row>
     <row r="9" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A9" s="42"/>
-      <c r="B9" s="38" t="s">
+      <c r="A9" s="44"/>
+      <c r="B9" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="40"/>
       <c r="AC9" s="22"/>
       <c r="AD9" s="19"/>
       <c r="AE9" s="19"/>
@@ -1981,12 +2026,12 @@
       <c r="AH9" s="23"/>
     </row>
     <row r="10" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A10" s="42"/>
-      <c r="B10" s="38" t="s">
+      <c r="A10" s="44"/>
+      <c r="B10" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="38"/>
-      <c r="D10" s="38"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
       <c r="S10" s="14"/>
       <c r="T10" s="15"/>
       <c r="U10" s="15"/>
@@ -1997,12 +2042,12 @@
       <c r="Z10" s="17"/>
     </row>
     <row r="11" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A11" s="42"/>
-      <c r="B11" s="38" t="s">
+      <c r="A11" s="44"/>
+      <c r="B11" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
       <c r="Z11" s="14"/>
       <c r="AA11" s="15"/>
       <c r="AB11" s="15"/>
@@ -2013,34 +2058,34 @@
       <c r="AG11" s="16"/>
     </row>
     <row r="12" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="42"/>
-      <c r="B12" s="38" t="s">
+      <c r="A12" s="44"/>
+      <c r="B12" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
       <c r="AF12" s="14"/>
       <c r="AG12" s="28"/>
       <c r="AH12" s="17"/>
     </row>
     <row r="13" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="42"/>
-      <c r="B13" s="38" t="s">
+      <c r="A13" s="44"/>
+      <c r="B13" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
       <c r="AG13" s="14"/>
       <c r="AH13" s="28"/>
       <c r="AI13" s="17"/>
     </row>
     <row r="14" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="42"/>
-      <c r="B14" s="38" t="s">
+      <c r="A14" s="44"/>
+      <c r="B14" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
       <c r="AH14" s="37"/>
       <c r="AI14" s="28"/>
       <c r="AJ14" s="28"/>
@@ -2051,14 +2096,15 @@
       <c r="AO14" s="28"/>
       <c r="AP14" s="28"/>
       <c r="AQ14" s="17"/>
+      <c r="BU14" s="47"/>
     </row>
     <row r="15" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="42"/>
-      <c r="B15" s="38" t="s">
+      <c r="A15" s="44"/>
+      <c r="B15" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
       <c r="AH15" s="22"/>
       <c r="AI15" s="19"/>
       <c r="AJ15" s="19"/>
@@ -2071,12 +2117,12 @@
       <c r="AQ15" s="23"/>
     </row>
     <row r="16" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="42"/>
-      <c r="B16" s="38" t="s">
+      <c r="A16" s="44"/>
+      <c r="B16" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
       <c r="AT16" s="29"/>
       <c r="AU16" s="31"/>
       <c r="AV16" s="31"/>
@@ -2085,12 +2131,12 @@
       <c r="AY16" s="30"/>
     </row>
     <row r="17" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="42"/>
-      <c r="B17" s="38" t="s">
+      <c r="A17" s="44"/>
+      <c r="B17" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
       <c r="AU17" s="29"/>
       <c r="AV17" s="31"/>
       <c r="AW17" s="31"/>
@@ -2100,12 +2146,12 @@
       <c r="BA17" s="30"/>
     </row>
     <row r="18" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="42"/>
-      <c r="B18" s="38" t="s">
+      <c r="A18" s="44"/>
+      <c r="B18" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
       <c r="BB18" s="14"/>
       <c r="BC18" s="15"/>
       <c r="BD18" s="15"/>
@@ -2115,12 +2161,12 @@
       <c r="BH18" s="16"/>
     </row>
     <row r="19" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="42"/>
-      <c r="B19" s="38" t="s">
+      <c r="A19" s="44"/>
+      <c r="B19" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
       <c r="BH19" s="29"/>
       <c r="BI19" s="31"/>
       <c r="BJ19" s="31"/>
@@ -2128,217 +2174,249 @@
       <c r="BL19" s="36"/>
     </row>
     <row r="20" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="42"/>
-      <c r="B20" s="39" t="s">
+      <c r="A20" s="44"/>
+      <c r="B20" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="40"/>
       <c r="BH20" s="33"/>
       <c r="BI20" s="34"/>
       <c r="BJ20" s="34"/>
       <c r="BK20" s="34"/>
       <c r="BL20" s="35"/>
-      <c r="BT20" s="44"/>
+      <c r="BT20" s="38"/>
     </row>
     <row r="21" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="42"/>
-      <c r="B21" s="38" t="s">
+      <c r="A21" s="44"/>
+      <c r="B21" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="40"/>
       <c r="BM21" s="29"/>
       <c r="BN21" s="31"/>
       <c r="BO21" s="31"/>
       <c r="BP21" s="30"/>
     </row>
-    <row r="22" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A22" s="42"/>
-      <c r="B22" s="38" t="s">
+    <row r="22" spans="1:102" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="44"/>
+      <c r="B22" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="BV22" s="11"/>
-      <c r="BW22" s="11"/>
-      <c r="BX22" s="11"/>
-      <c r="BY22" s="11"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+      <c r="BS22" s="22"/>
+      <c r="BT22" s="19"/>
+      <c r="BU22" s="19"/>
+      <c r="BV22" s="19"/>
+      <c r="BW22" s="19"/>
+      <c r="BX22" s="19"/>
+      <c r="BY22" s="19"/>
+      <c r="BZ22" s="19"/>
+      <c r="CA22" s="19"/>
+      <c r="CB22" s="19"/>
+      <c r="CC22" s="19"/>
+      <c r="CD22" s="46"/>
     </row>
     <row r="23" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A23" s="42"/>
-      <c r="B23" s="38" t="s">
+      <c r="A23" s="44"/>
+      <c r="B23" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="40"/>
+      <c r="D23" s="40"/>
+      <c r="BM23" s="33"/>
+      <c r="BN23" s="34"/>
+      <c r="BO23" s="34"/>
+      <c r="BP23" s="34"/>
+      <c r="BQ23" s="34"/>
+      <c r="BR23" s="34"/>
+      <c r="BS23" s="34"/>
+      <c r="BT23" s="34"/>
+      <c r="BU23" s="34"/>
+      <c r="BV23" s="34"/>
+      <c r="BW23" s="39"/>
+    </row>
+    <row r="24" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A24" s="44"/>
+      <c r="B24" s="40" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="BW24" s="33"/>
+      <c r="BX24" s="34"/>
+      <c r="BY24" s="34"/>
+      <c r="BZ24" s="34"/>
+      <c r="CA24" s="34"/>
+      <c r="CB24" s="34"/>
+      <c r="CC24" s="35"/>
+    </row>
+    <row r="25" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A25" s="44"/>
+      <c r="B25" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="CD25" s="11"/>
+      <c r="CE25" s="11"/>
+      <c r="CF25" s="11"/>
+      <c r="CG25" s="11"/>
+      <c r="CH25" s="11"/>
+      <c r="CI25" s="11"/>
+    </row>
+    <row r="26" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A26" s="44"/>
+      <c r="B26" s="40" t="s">
+        <v>41</v>
+      </c>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="CD26" s="13"/>
+      <c r="CE26" s="13"/>
+      <c r="CF26" s="13"/>
+      <c r="CG26" s="13"/>
+      <c r="CH26" s="13"/>
+      <c r="CI26" s="13"/>
+      <c r="CJ26" s="13"/>
+      <c r="CK26" s="13"/>
+      <c r="CL26" s="13"/>
+    </row>
+    <row r="27" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A27" s="44"/>
+      <c r="B27" s="40" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="CH27" s="11"/>
+      <c r="CI27" s="11"/>
+      <c r="CJ27" s="11"/>
+      <c r="CK27" s="11"/>
+      <c r="CL27" s="11"/>
+      <c r="CM27" s="11"/>
+    </row>
+    <row r="28" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A28" s="44"/>
+      <c r="B28" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="BM23" s="13"/>
-      <c r="BN23" s="13"/>
-      <c r="BO23" s="13"/>
-      <c r="BP23" s="13"/>
-      <c r="BQ23" s="13"/>
-      <c r="BR23" s="13"/>
-      <c r="BS23" s="13"/>
-      <c r="BT23" s="13"/>
-      <c r="BU23" s="13"/>
-      <c r="BV23" s="13"/>
-    </row>
-    <row r="24" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A24" s="42"/>
-      <c r="B24" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="BU24" s="13"/>
-      <c r="BV24" s="13"/>
-      <c r="BW24" s="13"/>
-      <c r="BX24" s="13"/>
-      <c r="BY24" s="13"/>
-      <c r="BZ24" s="13"/>
-      <c r="CA24" s="13"/>
-      <c r="CB24" s="13"/>
-      <c r="CC24" s="13"/>
-    </row>
-    <row r="25" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A25" s="42"/>
-      <c r="B25" s="38" t="s">
-        <v>39</v>
-      </c>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="BR25" s="27"/>
-      <c r="BS25" s="27"/>
-      <c r="BT25" s="27"/>
-      <c r="BU25" s="27"/>
-      <c r="BV25" s="27"/>
-      <c r="BW25" s="27"/>
-      <c r="BX25" s="27"/>
-      <c r="BY25" s="27"/>
-      <c r="BZ25" s="27"/>
-      <c r="CA25" s="27"/>
-      <c r="CB25" s="27"/>
-      <c r="CC25" s="27"/>
-      <c r="CD25" s="27"/>
-      <c r="CE25" s="27"/>
-      <c r="CF25" s="27"/>
-      <c r="CG25" s="27"/>
-      <c r="CH25" s="27"/>
-    </row>
-    <row r="26" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A26" s="42"/>
-      <c r="B26" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="C26" s="38"/>
-      <c r="D26" s="38"/>
-      <c r="BY26" s="27"/>
-      <c r="BZ26" s="27"/>
-      <c r="CA26" s="27"/>
-      <c r="CB26" s="27"/>
-      <c r="CC26" s="27"/>
-      <c r="CD26" s="27"/>
-      <c r="CE26" s="27"/>
-      <c r="CF26" s="27"/>
-      <c r="CG26" s="27"/>
-      <c r="CH26" s="27"/>
-      <c r="CI26" s="27"/>
-      <c r="CJ26" s="27"/>
-      <c r="CK26" s="27"/>
-      <c r="CL26" s="27"/>
-      <c r="CM26" s="27"/>
-      <c r="CN26" s="27"/>
-      <c r="CO26" s="27"/>
-      <c r="CP26" s="27"/>
-      <c r="CQ26" s="27"/>
-      <c r="CR26" s="27"/>
-      <c r="CS26" s="27"/>
-      <c r="CT26" s="27"/>
-      <c r="CU26" s="27"/>
-      <c r="CV26" s="27"/>
-      <c r="CW26" s="27"/>
-      <c r="CX26" s="27"/>
-    </row>
-    <row r="27" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A27" s="42"/>
-      <c r="B27" s="38" t="s">
+      <c r="C28" s="40"/>
+      <c r="D28" s="40"/>
+      <c r="CM28" s="11"/>
+      <c r="CN28" s="11"/>
+      <c r="CO28" s="11"/>
+      <c r="CP28" s="11"/>
+      <c r="CQ28" s="11"/>
+      <c r="CR28" s="11"/>
+      <c r="CS28" s="11"/>
+      <c r="CT28" s="11"/>
+    </row>
+    <row r="29" spans="1:102" x14ac:dyDescent="0.2">
+      <c r="A29" s="44"/>
+      <c r="B29" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="C27" s="38"/>
-      <c r="D27" s="38"/>
-    </row>
-    <row r="28" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A28" s="42"/>
-      <c r="B28" s="38"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="38"/>
-      <c r="CC28" s="11"/>
-      <c r="CD28" s="11"/>
-      <c r="CE28" s="11"/>
-      <c r="CF28" s="11"/>
-      <c r="CG28" s="11"/>
-    </row>
-    <row r="29" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A29" s="42"/>
-      <c r="B29" s="38"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="38"/>
+      <c r="C29" s="40"/>
+      <c r="D29" s="40"/>
+      <c r="CM29" s="13"/>
+      <c r="CN29" s="13"/>
+      <c r="CO29" s="13"/>
+      <c r="CP29" s="13"/>
+      <c r="CQ29" s="13"/>
+      <c r="CR29" s="13"/>
+      <c r="CS29" s="13"/>
+      <c r="CT29" s="13"/>
     </row>
     <row r="30" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A30" s="42"/>
+      <c r="A30" s="44"/>
+      <c r="B30" s="40" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" s="40"/>
+      <c r="D30" s="40"/>
+      <c r="CK30" s="48"/>
+      <c r="CL30" s="48"/>
+      <c r="CM30" s="48"/>
+      <c r="CN30" s="27"/>
+      <c r="CO30" s="27"/>
+      <c r="CP30" s="27"/>
+      <c r="CQ30" s="27"/>
+      <c r="CR30" s="27"/>
+      <c r="CS30" s="27"/>
+      <c r="CT30" s="27"/>
+      <c r="CU30" s="27"/>
+      <c r="CV30" s="27"/>
+      <c r="CW30" s="27"/>
+      <c r="CX30" s="27"/>
     </row>
     <row r="31" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A31" s="42"/>
+      <c r="A31" s="44"/>
+      <c r="B31" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="C31" s="40"/>
+      <c r="D31" s="40"/>
+      <c r="CR31" s="13"/>
+      <c r="CS31" s="13"/>
+      <c r="CT31" s="13"/>
+      <c r="CU31" s="13"/>
+      <c r="CV31" s="13"/>
+      <c r="CW31" s="13"/>
     </row>
     <row r="32" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="A32" s="42"/>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" s="42"/>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A34" s="42"/>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A35" s="42"/>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" s="42"/>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="44"/>
+      <c r="CE32" s="48"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="44"/>
+      <c r="C33" s="12"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="44"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="44"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="44"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="32"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="32"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="32"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="32"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="32"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="32"/>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="32"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="32"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="32"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="32"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" s="32"/>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="32"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
@@ -2402,7 +2480,8 @@
       <c r="A68" s="32"/>
     </row>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="39">
+    <mergeCell ref="B31:D31"/>
     <mergeCell ref="P2:R2"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="A1:CX1"/>
@@ -2424,22 +2503,23 @@
     <mergeCell ref="K2:M2"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B26:D26"/>
     <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B28:D28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>